<commit_message>
feat: bindings CIM-11 sur reaction.manifestation par type + 4 exemples
Ajoute 4 ValueSets dédiés (allergie : CIM-11 Chapitre 04 Bloc Affections
allergiques ou d'hypersensibilité ; hypersensibilité non allergique,
intolérance, idiosyncrasie : CIM-11 Chapitre 21), branchés en additional
binding extensible sur AllergyIntolerance.reaction.manifestation.

Ajoute 4 invariants (warning) indiquant quel ValueSet utiliser selon la
valeur de type (code natif pour allergy/intolerance, extension backport
R5 SNOMED CT pour hypersensibilité non allergique/idiosyncrasie).

Ajoute 3 nouveaux exemples (un par cas restant) et complète l'exemple
existant (cas allergie) avec un second coding CIM-11 sur manifestation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 5838d703275c3c66def6b92c9fbdd24460b9ba59
</commit_message>
<xml_diff>
--- a/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
+++ b/nr-doc-core-allergy-intolerance/ig/StructureDefinition-fr-core-allergy-intolerance.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-16T08:22:23+00:00</t>
+    <t>2026-09-16T15:48:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -273,7 +273,7 @@
   </si>
   <si>
     <t>ait-1:AllergyIntolerance.clinicalStatus SHALL be present if verificationStatus is not entered-in-error. {verificationStatus.coding.where(system = 'http://terminology.hl7.org/CodeSystem/allergyintolerance-verification' and code = 'entered-in-error').exists() or clinicalStatus.exists()}
-ait-2:AllergyIntolerance.clinicalStatus SHALL NOT be present if verification Status is entered-in-error {verificationStatus.coding.where(system = 'http://terminology.hl7.org/CodeSystem/allergyintolerance-verification' and code = 'entered-in-error').empty() or clinicalStatus.empty()}dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}</t>
+ait-2:AllergyIntolerance.clinicalStatus SHALL NOT be present if verification Status is entered-in-error {verificationStatus.coding.where(system = 'http://terminology.hl7.org/CodeSystem/allergyintolerance-verification' and code = 'entered-in-error').empty() or clinicalStatus.empty()}dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}fr-core-allergy-intolerance-1:Si type = allergie, les manifestations doivent être codées avec le ValueSet CIM-11 Chapitre 04, Bloc Affections allergiques ou d'hypersensibilité (fr-core-vs-allergyintolerance-manifestation-allergie). {type = 'allergy' implies reaction.manifestation.all(memberOf('https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-allergyintolerance-manifestation-allergie'))}fr-core-allergy-intolerance-2:Si type = hypersensibilité non allergique, les manifestations doivent être codées avec le ValueSet CIM-11 Chapitre 21 (fr-core-vs-allergyintolerance-manifestation-hypersensibilite). {type.extension('http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type').value.coding.exists(system = 'http://snomed.info/sct' and code = '609396006') implies reaction.manifestation.all(memberOf('https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-allergyintolerance-manifestation-hypersensibilite'))}fr-core-allergy-intolerance-3:Si type = intolérance, les manifestations doivent être codées avec le ValueSet CIM-11 Chapitre 21 (fr-core-vs-allergyintolerance-manifestation-intolerance). {type = 'intolerance' implies reaction.manifestation.all(memberOf('https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-allergyintolerance-manifestation-intolerance'))}fr-core-allergy-intolerance-4:Si type = idiosyncrasie, les manifestations doivent être codées avec le ValueSet CIM-11 Chapitre 21 (fr-core-vs-allergyintolerance-manifestation-idiosyncrasie). {type.extension('http://hl7.org/fhir/5.0/StructureDefinition/extension-AllergyIntolerance.type').value.coding.exists(system = 'http://snomed.info/sct' and code = '56840009') implies reaction.manifestation.all(memberOf('https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-allergyintolerance-manifestation-idiosyncrasie'))}</t>
   </si>
   <si>
     <t>Observation[classCode=OBS, moodCode=EVN]</t>

</xml_diff>